<commit_message>
Fix some card typos
</commit_message>
<xml_diff>
--- a/scripts/cards.xlsx
+++ b/scripts/cards.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="833">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1626" uniqueCount="833">
   <si>
     <t>id</t>
   </si>
@@ -1702,91 +1702,91 @@
     <t>Alongside the sharpnose sevengill (Heptranchias perlo), it's listed in the Guinness World Records as the fish with the most gill slits.</t>
   </si>
   <si>
+    <t>Common Bluestripe Snapper</t>
+  </si>
+  <si>
+    <t>Lutjanus kasmira</t>
+  </si>
+  <si>
+    <t>[BlueCoral][BlueCoral][BlueCoral]</t>
+  </si>
+  <si>
+    <t>It has a varied diet, feeding on fishes, shrimps, crabs, and crustaceans, as well as plant and algae material.</t>
+  </si>
+  <si>
+    <t>Daggertooth</t>
+  </si>
+  <si>
+    <t>Anotopterus pharao</t>
+  </si>
+  <si>
+    <t>[FishHatch] also, if [GreenCoral][GreenCoral][GreenCoral] in this dive site: [Discard]</t>
+  </si>
+  <si>
+    <t>Older daggertooth appear to turn black, lose their teeth, and migrate to deeper waters, possibly to reproduce.</t>
+  </si>
+  <si>
+    <t>Dusky Shark</t>
+  </si>
+  <si>
+    <t>Carcharhinus obscurus</t>
+  </si>
+  <si>
+    <t>[FreePlayFishFromHand][FishLengthMedium]only</t>
+  </si>
+  <si>
+    <t>It migrates hundreds to thousands of km to temperate waters in the summer and toward the equator in the winter.</t>
+  </si>
+  <si>
+    <t>Dwarf Lanternshark</t>
+  </si>
+  <si>
+    <t>Etmopterus perryi</t>
+  </si>
+  <si>
+    <t>[FreePlayFishFromHand][Bioluminescent] only</t>
+  </si>
+  <si>
+    <t>One of the smallest known sharks, the dwarf lanternshark's bioluminescent belly helps it blend in with sunlight from above.</t>
+  </si>
+  <si>
+    <t>Epaulette Shark</t>
+  </si>
+  <si>
+    <t>Hemiscyllium ocellatum</t>
+  </si>
+  <si>
+    <t>[BlueCoral][UnSchoolFish]</t>
+  </si>
+  <si>
+    <t>It can swim, but it mostly “walks” along coral reefs on its fins. It can even travel short distances over land.</t>
+  </si>
+  <si>
+    <t>Filetail Catshark</t>
+  </si>
+  <si>
+    <t>Parmaturus xaniurus</t>
+  </si>
+  <si>
+    <t>[FishFromHandConsume]</t>
+  </si>
+  <si>
+    <t>This catshark's common name comes from the toothlike projections on its skin.</t>
+  </si>
+  <si>
+    <t>Fire Dartfish</t>
+  </si>
+  <si>
+    <t>Nemateleotris magnifica</t>
+  </si>
+  <si>
+    <t>[PurpleCoral][PurpleCoral][PurpleCoral]</t>
+  </si>
+  <si>
+    <t>It usually hovers above its burrow, quick to dart inside. It flicks its long dorsal fin back and forth, perhaps as a signal.</t>
+  </si>
+  <si>
     <t>any:1</t>
-  </si>
-  <si>
-    <t>Common Bluestripe Snapper</t>
-  </si>
-  <si>
-    <t>Lutjanus kasmira</t>
-  </si>
-  <si>
-    <t>[BlueCoral][BlueCoral][BlueCoral]</t>
-  </si>
-  <si>
-    <t>It has a varied diet, feeding on fishes, shrimps, crabs, and crustaceans, as well as plant and algae material.</t>
-  </si>
-  <si>
-    <t>Daggertooth</t>
-  </si>
-  <si>
-    <t>Anotopterus pharao</t>
-  </si>
-  <si>
-    <t>[FishHatch] also, if [GreenCoral][GreenCoral][GreenCoral] in this dive site: [Discard]</t>
-  </si>
-  <si>
-    <t>Older daggertooth appear to turn black, lose their teeth, and migrate to deeper waters, possibly to reproduce.</t>
-  </si>
-  <si>
-    <t>Dusky Shark</t>
-  </si>
-  <si>
-    <t>Carcharhinus obscurus</t>
-  </si>
-  <si>
-    <t>[FreePlayFishFromHand][FishLengthMedium]only</t>
-  </si>
-  <si>
-    <t>It migrates hundreds to thousands of km to temperate waters in the summer and toward the equator in the winter.</t>
-  </si>
-  <si>
-    <t>Dwarf Lanternshark</t>
-  </si>
-  <si>
-    <t>Etmopterus perryi</t>
-  </si>
-  <si>
-    <t>[FreePlayFishFromHand][Bioluminescent] only</t>
-  </si>
-  <si>
-    <t>One of the smallest known sharks, the dwarf lanternshark's bioluminescent belly helps it blend in with sunlight from above.</t>
-  </si>
-  <si>
-    <t>Epaulette Shark</t>
-  </si>
-  <si>
-    <t>Hemiscyllium ocellatum</t>
-  </si>
-  <si>
-    <t>[BlueCoral][UnSchoolFish]</t>
-  </si>
-  <si>
-    <t>It can swim, but it mostly “walks” along coral reefs on its fins. It can even travel short distances over land.</t>
-  </si>
-  <si>
-    <t>Filetail Catshark</t>
-  </si>
-  <si>
-    <t>Parmaturus xaniurus</t>
-  </si>
-  <si>
-    <t>[FishFromHandConsume]</t>
-  </si>
-  <si>
-    <t>This catshark's common name comes from the toothlike projections on its skin.</t>
-  </si>
-  <si>
-    <t>Fire Dartfish</t>
-  </si>
-  <si>
-    <t>Nemateleotris magnifica</t>
-  </si>
-  <si>
-    <t>[PurpleCoral][PurpleCoral][PurpleCoral]</t>
-  </si>
-  <si>
-    <t>It usually hovers above its burrow, quick to dart inside. It flicks its long dorsal fin back and forth, perhaps as a signal.</t>
   </si>
   <si>
     <t>Flame Angelfish</t>
@@ -11101,9 +11101,7 @@
       <c r="U146" s="2">
         <v>0.0</v>
       </c>
-      <c r="V146" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="V146" s="2"/>
       <c r="W146" s="2" t="s">
         <v>558</v>
       </c>
@@ -11185,9 +11183,7 @@
       <c r="X147" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="Y147" s="2" t="s">
-        <v>563</v>
-      </c>
+      <c r="Y147" s="2"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="2">
@@ -11197,10 +11193,10 @@
         <v>25</v>
       </c>
       <c r="C148" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="D148" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="D148" s="2" t="s">
-        <v>565</v>
       </c>
       <c r="E148" s="2">
         <v>1.0</v>
@@ -11236,7 +11232,7 @@
         <v>28</v>
       </c>
       <c r="P148" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="Q148" s="2">
         <v>0.0</v>
@@ -11257,7 +11253,7 @@
         <v>78</v>
       </c>
       <c r="W148" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="X148" s="2" t="s">
         <v>522</v>
@@ -11272,10 +11268,10 @@
         <v>25</v>
       </c>
       <c r="C149" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="D149" s="2" t="s">
         <v>568</v>
-      </c>
-      <c r="D149" s="2" t="s">
-        <v>569</v>
       </c>
       <c r="E149" s="2">
         <v>0.0</v>
@@ -11311,7 +11307,7 @@
         <v>47</v>
       </c>
       <c r="P149" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="Q149" s="2">
         <v>0.0</v>
@@ -11332,7 +11328,7 @@
         <v>83</v>
       </c>
       <c r="W149" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="X149" s="2" t="s">
         <v>522</v>
@@ -11347,10 +11343,10 @@
         <v>25</v>
       </c>
       <c r="C150" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="D150" s="2" t="s">
         <v>572</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>573</v>
       </c>
       <c r="E150" s="2">
         <v>0.0</v>
@@ -11386,7 +11382,7 @@
         <v>28</v>
       </c>
       <c r="P150" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="Q150" s="2">
         <v>0.0</v>
@@ -11405,7 +11401,7 @@
       </c>
       <c r="V150" s="2"/>
       <c r="W150" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="X150" s="2" t="s">
         <v>522</v>
@@ -11420,10 +11416,10 @@
         <v>25</v>
       </c>
       <c r="C151" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="D151" s="2" t="s">
         <v>576</v>
-      </c>
-      <c r="D151" s="2" t="s">
-        <v>577</v>
       </c>
       <c r="E151" s="2">
         <v>2.0</v>
@@ -11459,7 +11455,7 @@
         <v>34</v>
       </c>
       <c r="P151" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="Q151" s="2">
         <v>1.0</v>
@@ -11478,7 +11474,7 @@
       </c>
       <c r="V151" s="2"/>
       <c r="W151" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="X151" s="2" t="s">
         <v>522</v>
@@ -11493,10 +11489,10 @@
         <v>25</v>
       </c>
       <c r="C152" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="D152" s="2" t="s">
         <v>580</v>
-      </c>
-      <c r="D152" s="2" t="s">
-        <v>581</v>
       </c>
       <c r="E152" s="2">
         <v>0.0</v>
@@ -11532,28 +11528,26 @@
         <v>34</v>
       </c>
       <c r="P152" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="Q152" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="R152" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="S152" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="T152" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="U152" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="V152" s="2"/>
+      <c r="W152" s="2" t="s">
         <v>582</v>
-      </c>
-      <c r="Q152" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="R152" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="S152" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="T152" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="U152" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="V152" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="W152" s="2" t="s">
-        <v>583</v>
       </c>
       <c r="X152" s="2" t="s">
         <v>522</v>
@@ -11570,10 +11564,10 @@
         <v>25</v>
       </c>
       <c r="C153" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="D153" s="2" t="s">
         <v>584</v>
-      </c>
-      <c r="D153" s="2" t="s">
-        <v>585</v>
       </c>
       <c r="E153" s="2">
         <v>3.0</v>
@@ -11609,7 +11603,7 @@
         <v>47</v>
       </c>
       <c r="P153" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="Q153" s="2">
         <v>0.0</v>
@@ -11628,7 +11622,7 @@
       </c>
       <c r="V153" s="2"/>
       <c r="W153" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="X153" s="2" t="s">
         <v>522</v>
@@ -11643,10 +11637,10 @@
         <v>25</v>
       </c>
       <c r="C154" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="D154" s="2" t="s">
         <v>588</v>
-      </c>
-      <c r="D154" s="2" t="s">
-        <v>589</v>
       </c>
       <c r="E154" s="2">
         <v>0.0</v>
@@ -11682,34 +11676,32 @@
         <v>28</v>
       </c>
       <c r="P154" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="Q154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="R154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="S154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="T154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="U154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="V154" s="2"/>
+      <c r="W154" s="2" t="s">
         <v>590</v>
-      </c>
-      <c r="Q154" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="R154" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="S154" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="T154" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="U154" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="V154" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="W154" s="2" t="s">
-        <v>591</v>
       </c>
       <c r="X154" s="2" t="s">
         <v>522</v>
       </c>
       <c r="Y154" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="155" ht="15.75" customHeight="1">
@@ -11776,7 +11768,9 @@
       <c r="U155" s="2">
         <v>0.0</v>
       </c>
-      <c r="V155" s="2"/>
+      <c r="V155" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="W155" s="2" t="s">
         <v>595</v>
       </c>
@@ -11851,7 +11845,9 @@
       <c r="U156" s="2">
         <v>1.0</v>
       </c>
-      <c r="V156" s="2"/>
+      <c r="V156" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="W156" s="2" t="s">
         <v>599</v>
       </c>
@@ -12445,9 +12441,7 @@
       <c r="U164" s="2">
         <v>0.0</v>
       </c>
-      <c r="V164" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="V164" s="2"/>
       <c r="W164" s="2" t="s">
         <v>632</v>
       </c>
@@ -13276,7 +13270,7 @@
         <v>522</v>
       </c>
       <c r="Y175" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="176" ht="15.75" customHeight="1">
@@ -13493,9 +13487,7 @@
       <c r="U178" s="2">
         <v>0.0</v>
       </c>
-      <c r="V178" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="V178" s="2"/>
       <c r="W178" s="2" t="s">
         <v>687</v>
       </c>
@@ -13801,7 +13793,7 @@
         <v>522</v>
       </c>
       <c r="Y182" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="183" ht="15.75" customHeight="1">
@@ -13876,7 +13868,7 @@
         <v>522</v>
       </c>
       <c r="Y183" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="184" ht="15.75" customHeight="1">
@@ -15293,7 +15285,9 @@
       <c r="U202" s="2">
         <v>0.0</v>
       </c>
-      <c r="V202" s="2"/>
+      <c r="V202" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="W202" s="2" t="s">
         <v>777</v>
       </c>
@@ -15676,7 +15670,7 @@
         <v>522</v>
       </c>
       <c r="Y207" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="208" ht="15.75" customHeight="1">
@@ -15824,7 +15818,7 @@
         <v>522</v>
       </c>
       <c r="Y209" s="2" t="s">
-        <v>563</v>
+        <v>591</v>
       </c>
     </row>
     <row r="210" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Fix a card typo
</commit_message>
<xml_diff>
--- a/scripts/cards.xlsx
+++ b/scripts/cards.xlsx
@@ -1861,8 +1861,7 @@
     <t>(all players) [PurpleCoral][PurpleCoral] [AllPlayers]</t>
   </si>
   <si>
-    <t>Sheltering by day in crevices up to  -50 meters deep, this nocturnal ambush predator hunts primarily by smell.</t>
+    <t>Sheltering by day in crevices up to 50 meters deep, this nocturnal ambush predator hunts primarily by smell.</t>
   </si>
   <si>
     <t>Goblin Shark</t>
@@ -12155,7 +12154,7 @@
         <v>0.0</v>
       </c>
       <c r="V160" s="2"/>
-      <c r="W160" s="2" t="s">
+      <c r="W160" s="3" t="s">
         <v>616</v>
       </c>
       <c r="X160" s="2" t="s">

</xml_diff>